<commit_message>
Add Adjustments sheet for manual projection haircuts
- New "Adjustments" sheet: Player | Adjust % | Reason; negative % scales
  a player's Proj 23 down (-20 => x0.8), applied after points are computed
- Seeded at -20%: Josh Jacobs (exempt list), Zach Charbonnet (PUP),
  George Kittle (Achilles), Rashod Bateman (legal)
- run_optimizer takes adjustments=; app shows the table and flags any
  adjusted player not in the active list

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fantasy_app.xlsx
+++ b/fantasy_app.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sleeper" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESPN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustments" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15586,4 +15587,95 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Adjust %</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Josh Jacobs</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Commissioner Exempt List - possible suspension (as of Sep 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Zach Charbonnet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>On PUP list - injury</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>George Kittle</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Recovering from torn Achilles - Week 1 status uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rashod Bateman</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Arrested (family violence) - possible suspension</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adjustments: drop Kittle & Bateman, add Puka Nacua
Per league call: Kittle not adjusted, Bateman cleared. Now -20% on
Josh Jacobs, Zach Charbonnet, Puka Nacua.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fantasy_app.xlsx
+++ b/fantasy_app.xlsx
@@ -15595,7 +15595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15648,7 +15648,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>George Kittle</t>
+          <t>Puka Nacua</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -15656,22 +15656,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Recovering from torn Achilles - Week 1 status uncertain</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Rashod Bateman</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-20</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Arrested (family violence) - possible suspension</t>
+          <t>Offseason legal matter - suspension risk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make adjustments editable in-app; restore Bateman
- Adjustments now render as an editable st.data_editor inside a
  collapsed expander: add/edit/delete rows per session, any player,
  +/- %, free-text Comment
- Workbook "Adjustments" sheet seeds the defaults (Reason -> Comment)
- Defaults: Josh Jacobs, Zach Charbonnet, Rashod Bateman, Puka Nacua
  at -20% (Kittle dropped earlier per league call)
- Session edits aren't persisted to the xlsx; edit the sheet for
  permanent defaults

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fantasy_app.xlsx
+++ b/fantasy_app.xlsx
@@ -15595,7 +15595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15611,7 +15611,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Commissioner Exempt List - possible suspension (as of Sep 2026)</t>
+          <t>Injury/legal: Commissioner Exempt List - possible suspension</t>
         </is>
       </c>
     </row>
@@ -15641,14 +15641,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>On PUP list - injury</t>
+          <t>Injury: on PUP list</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Puka Nacua</t>
+          <t>Rashod Bateman</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -15656,7 +15656,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Offseason legal matter - suspension risk</t>
+          <t>Legal: arrested (family violence) - possible suspension</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Puka Nacua</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Legal: offseason matter - suspension risk</t>
         </is>
       </c>
     </row>

</xml_diff>